<commit_message>
Complete V2 network diagrams, coupled system characteristics and engineering reports
</commit_message>
<xml_diff>
--- a/excel/Druckverlust_Netzwerk_V2.xlsx
+++ b/excel/Druckverlust_Netzwerk_V2.xlsx
@@ -23,6 +23,9 @@
     <sheet name="Netzwerk_Armaturen" sheetId="14" r:id="rId14"/>
     <sheet name="Netzwerk_Pumpe" sheetId="15" r:id="rId15"/>
     <sheet name="Netzwerk_Ergebnisse" sheetId="16" r:id="rId16"/>
+    <sheet name="Netzwerk_Diagramm" sheetId="17" r:id="rId17"/>
+    <sheet name="Netzwerk_Kennlinie" sheetId="18" r:id="rId18"/>
+    <sheet name="Netzwerk_Bericht" sheetId="19" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="ArmaturenTypen">'Armaturendatenbank'!$A$5:$A$16</definedName>
@@ -31,6 +34,7 @@
     <definedName name="NetzLeitungsIDs">tblNetzLeitungen[ID]</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">Blende_Standalone!$A$1:$H$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">Kv_Standalone!$A$1:$H$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="18">Netzwerk_Bericht!$A$1:$L$45</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">Systembericht!$A$1:$H$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -84,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="236">
   <si>
     <t>Rohrleitungs-Systemkennlinie</t>
   </si>
@@ -611,10 +615,10 @@
     <t>Geprueft durch: ____________________  Datum: ____________  Freigabe: ______________</t>
   </si>
   <si>
-    <t>Modus B | Netzwerk, Phasen 2 und 3</t>
-  </si>
-  <si>
-    <t>Eigene Stoffwerte und Eingaben, unabhaengig vom Einzelrohrmodus. VBA-Module aus vba/network zusaetzlich importieren. NetzwerkBerechnen / NetzwerkValidieren ueber Alt+F8. Diagramm und Netzwerkbericht folgen in spaeteren Phasen.</t>
+    <t>Modus B | Rohrleitungsnetzwerk</t>
+  </si>
+  <si>
+    <t>Eigene Stoffwerte und Eingaben, unabhaengig vom Einzelrohrmodus. VBA-Module aus vba/network zusaetzlich importieren. NetzwerkBerechnen / NetzwerkValidieren ueber Alt+F8. NetzwerkEinrichtung legt Schaltflaechen fuer Schema, Kennlinie und Bericht an.</t>
   </si>
   <si>
     <t>Iterationslimit</t>
@@ -629,6 +633,24 @@
     <t>Fiktives laminares Beispiel. Externer Zufluss positiv, Entnahme negativ. Fester Absolutdruck und externe Flussvorgabe am selben Knoten werden abgelehnt. Druckknoten liefern den berechneten Reservoir-Zu-/Abfluss. Offener Auslass: lokalen Atmosphaerendruck explizit eingeben.</t>
   </si>
   <si>
+    <t>Einspeiseknoten / Pumpen-Druckstutzen</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Kennlinie Qmin m3/h</t>
+  </si>
+  <si>
+    <t>Kennlinie Qmax m3/h</t>
+  </si>
+  <si>
+    <t>Kennlinienpunkte</t>
+  </si>
+  <si>
+    <t>Kennlinie ohne Pumpe: Absolutdruck am ausgewaehlten Port bei vorgegebenem Q. Mit Pumpe: Einspeisung=Endknoten der Pumpenleitung; erforderliche Pumpen-dp bei festem Pumpen-Q. Andere Randbedingungen bleiben unveraendert. Bei nicht eindeutiger Kurve Netzwerkbetriebspunkt waehlen.</t>
+  </si>
+  <si>
     <t>Netzwerk_Knoten</t>
   </si>
   <si>
@@ -656,9 +678,6 @@
     <t>Y optional</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>Quelle</t>
   </si>
   <si>
@@ -756,6 +775,27 @@
   </si>
   <si>
     <t>Ergebnisse werden nur bei konvergierten und geprueften Bilanzen geschrieben.</t>
+  </si>
+  <si>
+    <t>Hydraulisches Netz | Schema</t>
+  </si>
+  <si>
+    <t>NICHT BERECHNET | NetzwerkBerechnen erzeugt eigene Shapes.</t>
+  </si>
+  <si>
+    <t>X/Y in Punkten relativ zum Schema; manuell verschieben, dann NetzwerkPositionenSpeichern. Nicht massstaeblich.</t>
+  </si>
+  <si>
+    <t>Netzwerk-Systemkennlinie</t>
+  </si>
+  <si>
+    <t>NICHT BERECHNET</t>
+  </si>
+  <si>
+    <t>Rohrleitungsnetz | Engineering-Bericht</t>
+  </si>
+  <si>
+    <t>NICHT BERECHNET | NetzwerkBerichtErstellen</t>
   </si>
 </sst>
 </file>
@@ -2792,7 +2832,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="48.7109375" customWidth="1"/>
@@ -2911,11 +2951,83 @@
       <c r="E15" s="19"/>
       <c r="F15" s="19"/>
     </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>181</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>183</v>
+      </c>
+      <c r="B18" s="20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B19" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>185</v>
+      </c>
+      <c r="B20" s="20">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="19"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="19"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="19"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:F3"/>
     <mergeCell ref="A12:F15"/>
+    <mergeCell ref="A23:F26"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17">
+      <formula1>NetzKnotenIDs</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2930,49 +3042,49 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="18" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="19" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B4" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="E4" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="F4" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="G4" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="H4" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="20" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D5" s="20">
         <v>0</v>
@@ -2986,13 +3098,13 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="20" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D6" s="20">
         <v>0</v>
@@ -3004,13 +3116,13 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="20" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="D7" s="20">
         <v>0</v>
@@ -3045,58 +3157,58 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="18" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="19" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B4" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C4" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="E4" t="s">
         <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G4" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="H4" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="I4" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="J4" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="20" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E5" s="20">
         <v>50</v>
@@ -3119,16 +3231,16 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="20" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E6" s="20">
         <v>50</v>
@@ -3178,20 +3290,20 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="18" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="19" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -3203,24 +3315,24 @@
         <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="G4" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="H4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="I4" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="J4" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="20" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>44</v>
@@ -3271,20 +3383,20 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="18" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="19" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B4" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -3353,21 +3465,174 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="18" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="19" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="19" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="20" customHeight="1"/>
+  <cols>
+    <col min="1" max="52" width="13.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="20" customHeight="1">
+      <c r="A1" s="18" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="20" customHeight="1">
+      <c r="A2" s="19" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="20" customHeight="1">
+      <c r="A3" s="19" t="s">
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="5" width="22.7109375" customWidth="1"/>
+    <col min="7" max="52" width="14.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="18" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="19" t="s">
+        <v>233</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:U6"/>
+  <sheetFormatPr defaultRowHeight="16" customHeight="1"/>
+  <cols>
+    <col min="1" max="12" width="9.7109375" customWidth="1"/>
+    <col min="14" max="21" width="16.7109375" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="16" customHeight="1">
+      <c r="A1" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+    </row>
+    <row r="2" spans="1:12" ht="16" customHeight="1">
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+    </row>
+    <row r="3" spans="1:12" ht="16" customHeight="1">
+      <c r="A3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" t="s">
+        <v>109</v>
+      </c>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+    </row>
+    <row r="4" spans="1:12" ht="16" customHeight="1">
+      <c r="A4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" t="s">
+        <v>110</v>
+      </c>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+    </row>
+    <row r="6" spans="1:12" ht="16" customHeight="1">
+      <c r="A6" s="19" t="s">
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="H4:L4"/>
+  </mergeCells>
+  <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.35" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="85" orientation="landscape"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BDruckverlust | Netzwerk&amp;B</oddHeader>
+    <oddFooter>&amp;L&amp;D&amp;RSeite &amp;P von &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 

</xml_diff>